<commit_message>
Ground Sprite 추가 & 시작할 때 Sprite 로드
</commit_message>
<xml_diff>
--- a/Assets/100_Data/XlsxFiles/Ground_Data.xlsx
+++ b/Assets/100_Data/XlsxFiles/Ground_Data.xlsx
@@ -19,18 +19,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
   <si>
     <t>HP</t>
-  </si>
-  <si>
-    <t>Light_Brown[Light_Brown]</t>
-  </si>
-  <si>
-    <t>Deep_Brown[Deep_Brown]</t>
-  </si>
-  <si>
-    <t>Lava_Earth[Lava_Earth]</t>
   </si>
   <si>
     <t>Id</t>
@@ -75,6 +66,10 @@
   </si>
   <si>
     <t>1001;1003;1005</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ground1</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1022,25 +1017,25 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
@@ -1048,7 +1043,7 @@
         <v>5001</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -1063,7 +1058,7 @@
         <v>1001</v>
       </c>
       <c r="G2" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -1071,7 +1066,7 @@
         <v>5002</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C3">
         <v>6</v>
@@ -1083,10 +1078,10 @@
         <v>5</v>
       </c>
       <c r="F3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G3" t="s">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -1094,7 +1089,7 @@
         <v>5003</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C4">
         <v>11</v>
@@ -1106,10 +1101,10 @@
         <v>5</v>
       </c>
       <c r="F4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G4" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -1117,7 +1112,7 @@
         <v>5004</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C5">
         <v>16</v>
@@ -1132,7 +1127,7 @@
         <v>1007</v>
       </c>
       <c r="G5" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>